<commit_message>
minor data dictionar changes
</commit_message>
<xml_diff>
--- a/www/data-entry-template/GLATAR_data_entry_template_v17_long.xlsx
+++ b/www/data-entry-template/GLATAR_data_entry_template_v17_long.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benhlina/Library/CloudStorage/Dropbox/GitHub/GLATAR-App/www/data-entry-template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{499185CE-00B5-1B42-84BE-CC7F8952EE4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04AB0F68-1943-7547-9CE0-DB5C1CF86938}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="640" windowWidth="34560" windowHeight="19460" xr2:uid="{DE6F8925-643B-304C-8933-23D4A9123DA3}"/>
+    <workbookView xWindow="-25580" yWindow="1720" windowWidth="25600" windowHeight="19460" xr2:uid="{DE6F8925-643B-304C-8933-23D4A9123DA3}"/>
   </bookViews>
   <sheets>
     <sheet name="data_dictionary" sheetId="1" r:id="rId1"/>
@@ -1087,9 +1087,6 @@
     <t>amino_acid_measurement</t>
   </si>
   <si>
-    <t>as in: 2.4 ‰; format; integer</t>
-  </si>
-  <si>
     <t>Percent amino acid of a sample</t>
   </si>
   <si>
@@ -1100,9 +1097,6 @@
   </si>
   <si>
     <t>amino_acid_type</t>
-  </si>
-  <si>
-    <t>as in: Alanine: format; character</t>
   </si>
   <si>
     <t>Type of amino acid</t>
@@ -1117,16 +1111,10 @@
     <t>mercury_ppm</t>
   </si>
   <si>
-    <t>as in: 0.14; format: integer</t>
-  </si>
-  <si>
     <t>Mercury measurement</t>
   </si>
   <si>
     <t>mercury_type</t>
-  </si>
-  <si>
-    <t>as in: methylmercury: format; character</t>
   </si>
   <si>
     <t xml:space="preserve">Type of mercury </t>
@@ -1139,9 +1127,6 @@
   </si>
   <si>
     <t>pcb_congener_ng_g</t>
-  </si>
-  <si>
-    <t>as in: 0.20; format: integer</t>
   </si>
   <si>
     <t>Polychlorimated biphenols (PCB) congener measurement</t>
@@ -1216,9 +1201,6 @@
     <t>as in: Th (free thiamine); format: character</t>
   </si>
   <si>
-    <t>as in: 0.12; fromat: numeric</t>
-  </si>
-  <si>
     <t>as in: 0.6; format: numeric</t>
   </si>
   <si>
@@ -1229,6 +1211,24 @@
   </si>
   <si>
     <t>Standard deviation of Thiaminase activity if reported as mean</t>
+  </si>
+  <si>
+    <t>as in: Alanine; format: character</t>
+  </si>
+  <si>
+    <t>as in: methylmercury; format: character</t>
+  </si>
+  <si>
+    <t>as in: 0.14; format: numeric</t>
+  </si>
+  <si>
+    <t>as in: 0.20; format: numeric</t>
+  </si>
+  <si>
+    <t>as in: 2.4 ‰; format: numeric</t>
+  </si>
+  <si>
+    <t>as in: 0.12; format: numeric</t>
   </si>
 </sst>
 </file>
@@ -1456,7 +1456,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1549,18 +1549,10 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1583,6 +1575,13 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1935,20 +1934,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="48" t="s">
         <v>211</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
     </row>
     <row r="2" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="48" t="s">
         <v>192</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="21" t="s">
@@ -2003,7 +2002,7 @@
         <v>171</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -2017,7 +2016,7 @@
         <v>66</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="28" x14ac:dyDescent="0.2">
@@ -2059,7 +2058,7 @@
         <v>171</v>
       </c>
       <c r="D11" s="24" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
@@ -2325,7 +2324,7 @@
         <v>160</v>
       </c>
       <c r="D30" s="30" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
@@ -2406,7 +2405,7 @@
         <v>186</v>
       </c>
       <c r="C36" s="30" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="D36" s="33" t="s">
         <v>214</v>
@@ -2521,7 +2520,7 @@
         <v>79</v>
       </c>
       <c r="D44" s="30" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
@@ -2644,10 +2643,10 @@
         <v>109</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
@@ -2731,7 +2730,7 @@
         <v>180</v>
       </c>
       <c r="D59" s="30" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
@@ -3022,10 +3021,10 @@
         <v>249</v>
       </c>
       <c r="C80" s="30" t="s">
+        <v>296</v>
+      </c>
+      <c r="D80" s="33" t="s">
         <v>250</v>
-      </c>
-      <c r="D80" s="33" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="81" spans="1:4" ht="42" x14ac:dyDescent="0.2">
@@ -3033,13 +3032,13 @@
         <v>248</v>
       </c>
       <c r="B81" s="30" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C81" s="30" t="s">
         <v>243</v>
       </c>
       <c r="D81" s="33" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.2">
@@ -3047,153 +3046,153 @@
         <v>248</v>
       </c>
       <c r="B82" s="30" t="s">
+        <v>253</v>
+      </c>
+      <c r="C82" s="30" t="s">
+        <v>292</v>
+      </c>
+      <c r="D82" s="33" t="s">
         <v>254</v>
-      </c>
-      <c r="C82" s="30" t="s">
-        <v>255</v>
-      </c>
-      <c r="D82" s="33" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A83" s="30" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="B83" s="30" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C83" s="30" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="D83" s="30" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="84" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A84" s="30" t="s">
-        <v>275</v>
-      </c>
-      <c r="B84" s="43" t="s">
-        <v>286</v>
+        <v>270</v>
+      </c>
+      <c r="B84" s="40" t="s">
+        <v>281</v>
       </c>
       <c r="C84" s="30" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="D84" s="33" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
     </row>
     <row r="85" spans="1:4" ht="42" x14ac:dyDescent="0.2">
       <c r="A85" s="30" t="s">
-        <v>275</v>
-      </c>
-      <c r="B85" s="43" t="s">
+        <v>270</v>
+      </c>
+      <c r="B85" s="40" t="s">
+        <v>280</v>
+      </c>
+      <c r="C85" s="30" t="s">
+        <v>287</v>
+      </c>
+      <c r="D85" s="33" t="s">
         <v>285</v>
-      </c>
-      <c r="C85" s="30" t="s">
-        <v>292</v>
-      </c>
-      <c r="D85" s="33" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A86" s="30" t="s">
-        <v>275</v>
-      </c>
-      <c r="B86" s="43" t="s">
-        <v>287</v>
+        <v>270</v>
+      </c>
+      <c r="B86" s="40" t="s">
+        <v>282</v>
       </c>
       <c r="C86" s="30" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="D86" s="30" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A87" s="30" t="s">
-        <v>275</v>
-      </c>
-      <c r="B87" s="43" t="s">
-        <v>288</v>
+        <v>270</v>
+      </c>
+      <c r="B87" s="40" t="s">
+        <v>283</v>
       </c>
       <c r="C87" s="30" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="D87" s="30" t="s">
-        <v>297</v>
+        <v>291</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A88" s="30" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="B88" s="30" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="C88" s="30" t="s">
-        <v>260</v>
+        <v>294</v>
       </c>
       <c r="D88" s="30" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A89" s="30" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="B89" s="30" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="C89" s="30" t="s">
-        <v>263</v>
+        <v>293</v>
       </c>
       <c r="D89" s="30" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A90" s="30" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="B90" s="30" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="C90" s="30" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="D90" s="30" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A91" s="30" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="B91" s="30" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="C91" s="30" t="s">
-        <v>268</v>
+        <v>295</v>
       </c>
       <c r="D91" s="30" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A92" s="30" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="B92" s="30" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="C92" s="30" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="D92" s="30" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -3217,27 +3216,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="49" t="s">
         <v>202</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
       <c r="D1" s="10" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="49" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42"/>
+      <c r="B2" s="50"/>
+      <c r="C2" s="50"/>
       <c r="D2" s="11"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="41"/>
-      <c r="B3" s="41"/>
-      <c r="C3" s="41"/>
+      <c r="A3" s="49"/>
+      <c r="B3" s="49"/>
+      <c r="C3" s="49"/>
       <c r="D3" s="11" t="s">
         <v>206</v>
       </c>
@@ -3283,27 +3282,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="49" t="s">
         <v>190</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
       <c r="D1" s="10" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="49" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42"/>
+      <c r="B2" s="50"/>
+      <c r="C2" s="50"/>
       <c r="D2" s="11"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A3" s="41"/>
-      <c r="B3" s="42"/>
-      <c r="C3" s="42"/>
+      <c r="A3" s="49"/>
+      <c r="B3" s="50"/>
+      <c r="C3" s="50"/>
       <c r="D3" s="11" t="s">
         <v>25</v>
       </c>
@@ -44261,7 +44260,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED99CF4A-5D49-794D-A1CB-3B08F37AF445}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:BT29"/>
+  <dimension ref="A1:BT22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="20.5" customWidth="1"/>
@@ -44313,27 +44312,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:72" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="49" t="s">
         <v>189</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
       <c r="D1" s="5" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="2" spans="1:72" x14ac:dyDescent="0.2">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="49" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42"/>
+      <c r="B2" s="50"/>
+      <c r="C2" s="50"/>
       <c r="D2" s="6"/>
     </row>
     <row r="3" spans="1:72" x14ac:dyDescent="0.2">
-      <c r="A3" s="41"/>
-      <c r="B3" s="42"/>
-      <c r="C3" s="42"/>
+      <c r="A3" s="49"/>
+      <c r="B3" s="50"/>
+      <c r="C3" s="50"/>
       <c r="D3" s="6" t="s">
         <v>25</v>
       </c>
@@ -44370,14 +44369,14 @@
       <c r="BI4" s="38"/>
       <c r="BJ4" s="38"/>
       <c r="BK4" s="38" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="BL4" s="38"/>
       <c r="BM4" s="38"/>
       <c r="BN4" s="38"/>
       <c r="BO4" s="38"/>
       <c r="BP4" s="38" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="BQ4" s="38"/>
       <c r="BR4" s="38"/>
@@ -44385,16 +44384,16 @@
       <c r="BT4" s="38"/>
     </row>
     <row r="5" spans="1:72" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="46" t="s">
+      <c r="A5" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="46" t="s">
+      <c r="B5" s="42" t="s">
         <v>80</v>
       </c>
       <c r="C5" s="36" t="s">
         <v>194</v>
       </c>
-      <c r="D5" s="47" t="s">
+      <c r="D5" s="43" t="s">
         <v>199</v>
       </c>
       <c r="E5" s="36" t="s">
@@ -44406,10 +44405,10 @@
       <c r="G5" s="36" t="s">
         <v>135</v>
       </c>
-      <c r="H5" s="48" t="s">
+      <c r="H5" s="44" t="s">
         <v>195</v>
       </c>
-      <c r="I5" s="48" t="s">
+      <c r="I5" s="44" t="s">
         <v>193</v>
       </c>
       <c r="J5" s="36" t="s">
@@ -44424,7 +44423,7 @@
       <c r="M5" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="N5" s="48" t="s">
+      <c r="N5" s="44" t="s">
         <v>13</v>
       </c>
       <c r="O5" s="36" t="s">
@@ -44442,22 +44441,22 @@
       <c r="S5" s="36" t="s">
         <v>201</v>
       </c>
-      <c r="T5" s="49" t="s">
+      <c r="T5" s="45" t="s">
         <v>72</v>
       </c>
-      <c r="U5" s="49" t="s">
+      <c r="U5" s="45" t="s">
         <v>73</v>
       </c>
-      <c r="V5" s="48" t="s">
+      <c r="V5" s="44" t="s">
         <v>9</v>
       </c>
-      <c r="W5" s="50" t="s">
+      <c r="W5" s="46" t="s">
         <v>71</v>
       </c>
-      <c r="X5" s="49" t="s">
+      <c r="X5" s="45" t="s">
         <v>122</v>
       </c>
-      <c r="Y5" s="48" t="s">
+      <c r="Y5" s="44" t="s">
         <v>17</v>
       </c>
       <c r="Z5" s="36" t="s">
@@ -44469,16 +44468,16 @@
       <c r="AB5" s="36" t="s">
         <v>21</v>
       </c>
-      <c r="AC5" s="51" t="s">
+      <c r="AC5" s="47" t="s">
         <v>197</v>
       </c>
-      <c r="AD5" s="51" t="s">
+      <c r="AD5" s="47" t="s">
         <v>198</v>
       </c>
-      <c r="AE5" s="51" t="s">
+      <c r="AE5" s="47" t="s">
         <v>67</v>
       </c>
-      <c r="AF5" s="51" t="s">
+      <c r="AF5" s="47" t="s">
         <v>109</v>
       </c>
       <c r="AG5" s="36" t="s">
@@ -44493,16 +44492,16 @@
       <c r="AJ5" s="36" t="s">
         <v>116</v>
       </c>
-      <c r="AK5" s="49" t="s">
+      <c r="AK5" s="45" t="s">
         <v>139</v>
       </c>
-      <c r="AL5" s="49" t="s">
+      <c r="AL5" s="45" t="s">
         <v>140</v>
       </c>
-      <c r="AM5" s="49" t="s">
+      <c r="AM5" s="45" t="s">
         <v>143</v>
       </c>
-      <c r="AN5" s="49" t="s">
+      <c r="AN5" s="45" t="s">
         <v>144</v>
       </c>
       <c r="AO5" s="36" t="s">
@@ -44566,92 +44565,53 @@
         <v>249</v>
       </c>
       <c r="BI5" s="39" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="BJ5" s="39" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="BK5" s="39" t="s">
+        <v>255</v>
+      </c>
+      <c r="BL5" s="39" t="s">
+        <v>281</v>
+      </c>
+      <c r="BM5" s="39" t="s">
+        <v>280</v>
+      </c>
+      <c r="BN5" s="39" t="s">
+        <v>282</v>
+      </c>
+      <c r="BO5" s="39" t="s">
+        <v>283</v>
+      </c>
+      <c r="BP5" s="39" t="s">
         <v>257</v>
       </c>
-      <c r="BL5" s="39" t="s">
-        <v>286</v>
-      </c>
-      <c r="BM5" s="39" t="s">
-        <v>285</v>
-      </c>
-      <c r="BN5" s="39" t="s">
-        <v>287</v>
-      </c>
-      <c r="BO5" s="39" t="s">
-        <v>288</v>
-      </c>
-      <c r="BP5" s="39" t="s">
+      <c r="BQ5" s="39" t="s">
         <v>259</v>
       </c>
-      <c r="BQ5" s="39" t="s">
-        <v>262</v>
-      </c>
       <c r="BR5" s="39" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="BS5" s="39" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="BT5" s="39" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="13" spans="1:72" x14ac:dyDescent="0.2">
-      <c r="BK13" s="44"/>
-    </row>
-    <row r="14" spans="1:72" x14ac:dyDescent="0.2">
-      <c r="BK14" s="44"/>
-    </row>
-    <row r="15" spans="1:72" x14ac:dyDescent="0.2">
-      <c r="BK15" s="44"/>
-    </row>
-    <row r="16" spans="1:72" x14ac:dyDescent="0.2">
-      <c r="BK16" s="44"/>
-    </row>
-    <row r="17" spans="63:63" x14ac:dyDescent="0.2">
-      <c r="BK17" s="44"/>
-    </row>
-    <row r="18" spans="63:63" x14ac:dyDescent="0.2">
-      <c r="BK18" s="44"/>
+        <v>265</v>
+      </c>
     </row>
     <row r="19" spans="63:63" x14ac:dyDescent="0.2">
-      <c r="BK19" s="45"/>
+      <c r="BK19" s="41"/>
     </row>
     <row r="20" spans="63:63" x14ac:dyDescent="0.2">
-      <c r="BK20" s="45"/>
+      <c r="BK20" s="41"/>
     </row>
     <row r="21" spans="63:63" x14ac:dyDescent="0.2">
-      <c r="BK21" s="45"/>
+      <c r="BK21" s="41"/>
     </row>
     <row r="22" spans="63:63" x14ac:dyDescent="0.2">
-      <c r="BK22" s="45"/>
-    </row>
-    <row r="23" spans="63:63" x14ac:dyDescent="0.2">
-      <c r="BK23" s="44"/>
-    </row>
-    <row r="24" spans="63:63" x14ac:dyDescent="0.2">
-      <c r="BK24" s="44"/>
-    </row>
-    <row r="25" spans="63:63" x14ac:dyDescent="0.2">
-      <c r="BK25" s="44"/>
-    </row>
-    <row r="26" spans="63:63" x14ac:dyDescent="0.2">
-      <c r="BK26" s="44"/>
-    </row>
-    <row r="27" spans="63:63" x14ac:dyDescent="0.2">
-      <c r="BK27" s="44"/>
-    </row>
-    <row r="28" spans="63:63" x14ac:dyDescent="0.2">
-      <c r="BK28" s="44"/>
-    </row>
-    <row r="29" spans="63:63" x14ac:dyDescent="0.2">
-      <c r="BK29" s="44"/>
+      <c r="BK22" s="41"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1"/>

</xml_diff>